<commit_message>
revised_3_2_2: add variable labels, fix window sizes, and improve pipeline robustness
- Add comprehensive variable labels to all 116 final output variables
- Fix weather time windows (6h/12h/24h) to correct sizes (12/24/48 hours)
- Fix closure_frequency.csv import to handle title row
- Add v3 port-specific open probability
- Preserve Stata variable labels through Python roundtrip
</commit_message>
<xml_diff>
--- a/logs/duplicate_transactions_real.xlsx
+++ b/logs/duplicate_transactions_real.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:T22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -460,65 +460,75 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>start_mins</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>enddate</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>endhour</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>end_mins</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>port</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>supplier_n</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>supplier1</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>supplier2</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>supplier3</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>supplier4</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>supplier5</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>supplier6</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>supplier7</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>supplier8</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>supplier9</t>
         </is>
@@ -540,39 +550,45 @@
         <v>44979</v>
       </c>
       <c r="E2" t="n">
-        <v>11</v>
-      </c>
-      <c r="F2" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>44980</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>15</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="K2" t="n">
         <v>2</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Hongheng169</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>An Tong 27</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -590,24 +606,28 @@
         <v>44979</v>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
-      </c>
-      <c r="F3" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>44980</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>15</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="n">
+        <v>21</v>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="K3" t="n">
         <v>0</v>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
@@ -615,6 +635,8 @@
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -632,39 +654,45 @@
         <v>44979</v>
       </c>
       <c r="E4" t="n">
-        <v>11</v>
-      </c>
-      <c r="F4" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F4" t="n">
+        <v>35</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>44980</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>15</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="K4" t="n">
         <v>2</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Hongheng169</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>An Tong 27</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -684,37 +712,43 @@
       <c r="E5" t="n">
         <v>12</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>45028</v>
       </c>
-      <c r="G5" t="n">
-        <v>10</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" t="n">
+        <v>9</v>
+      </c>
+      <c r="I5" t="n">
+        <v>41</v>
+      </c>
+      <c r="J5" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="K5" t="n">
         <v>2</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Chaoyang301</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Fu Jie 168</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -734,22 +768,26 @@
       <c r="E6" t="n">
         <v>12</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>45028</v>
       </c>
-      <c r="G6" t="n">
-        <v>10</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" t="n">
+        <v>9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>41</v>
+      </c>
+      <c r="J6" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="K6" t="n">
         <v>0</v>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
@@ -757,6 +795,8 @@
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+      <c r="T6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -776,37 +816,43 @@
       <c r="E7" t="n">
         <v>12</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>45028</v>
       </c>
-      <c r="G7" t="n">
-        <v>10</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" t="n">
+        <v>9</v>
+      </c>
+      <c r="I7" t="n">
+        <v>41</v>
+      </c>
+      <c r="J7" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="K7" t="n">
         <v>2</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Chaoyang301</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Fu Jie 168</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -824,35 +870,41 @@
         <v>45065</v>
       </c>
       <c r="E8" t="n">
-        <v>13</v>
-      </c>
-      <c r="F8" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>39</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>45066</v>
       </c>
-      <c r="G8" t="n">
-        <v>12</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="H8" t="n">
+        <v>11</v>
+      </c>
+      <c r="I8" t="n">
+        <v>39</v>
+      </c>
+      <c r="J8" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="K8" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Chaoyang301</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
+      <c r="T8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -870,24 +922,28 @@
         <v>45065</v>
       </c>
       <c r="E9" t="n">
-        <v>13</v>
-      </c>
-      <c r="F9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>39</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>45066</v>
       </c>
-      <c r="G9" t="n">
-        <v>12</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="H9" t="n">
+        <v>11</v>
+      </c>
+      <c r="I9" t="n">
+        <v>39</v>
+      </c>
+      <c r="J9" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="K9" t="n">
         <v>0</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -895,6 +951,8 @@
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
+      <c r="T9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -912,35 +970,41 @@
         <v>45065</v>
       </c>
       <c r="E10" t="n">
-        <v>13</v>
-      </c>
-      <c r="F10" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" t="n">
+        <v>39</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>45066</v>
       </c>
-      <c r="G10" t="n">
-        <v>12</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="H10" t="n">
+        <v>11</v>
+      </c>
+      <c r="I10" t="n">
+        <v>39</v>
+      </c>
+      <c r="J10" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="K10" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Chaoyang301</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -958,39 +1022,45 @@
         <v>45403</v>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
-      </c>
-      <c r="F11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F11" t="n">
+        <v>44</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>45403</v>
       </c>
-      <c r="G11" t="n">
+      <c r="H11" t="n">
         <v>15</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="n">
+        <v>16</v>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="K11" t="n">
         <v>2</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Hui Chen 118</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1008,39 +1078,45 @@
         <v>45403</v>
       </c>
       <c r="E12" t="n">
-        <v>7</v>
-      </c>
-      <c r="F12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>44</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>45403</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>15</v>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="n">
+        <v>16</v>
+      </c>
+      <c r="J12" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="K12" t="n">
         <v>2</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Hui Chen 118</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1060,33 +1136,39 @@
       <c r="E13" t="n">
         <v>19</v>
       </c>
-      <c r="F13" s="2" t="n">
+      <c r="F13" t="n">
+        <v>17</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>45262</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>11</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>条帚门</t>
-        </is>
       </c>
       <c r="I13" t="n">
         <v>1</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
+          <t>条帚门</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1106,33 +1188,39 @@
       <c r="E14" t="n">
         <v>19</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" t="n">
+        <v>17</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>45262</v>
       </c>
-      <c r="G14" t="n">
+      <c r="H14" t="n">
         <v>11</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>条帚门</t>
-        </is>
       </c>
       <c r="I14" t="n">
         <v>1</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
+          <t>条帚门</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
+      <c r="T14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1150,39 +1238,45 @@
         <v>45386</v>
       </c>
       <c r="E15" t="n">
-        <v>11</v>
-      </c>
-      <c r="F15" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F15" t="n">
+        <v>59</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>45388</v>
       </c>
-      <c r="G15" t="n">
+      <c r="H15" t="n">
         <v>7</v>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="n">
+        <v>17</v>
+      </c>
+      <c r="J15" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I15" t="n">
+      <c r="K15" t="n">
         <v>2</v>
       </c>
-      <c r="J15" t="inlineStr">
+      <c r="L15" t="inlineStr">
         <is>
           <t>Shun Ping 17</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
+      <c r="M15" t="inlineStr">
         <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+      <c r="T15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1200,39 +1294,45 @@
         <v>45386</v>
       </c>
       <c r="E16" t="n">
-        <v>11</v>
-      </c>
-      <c r="F16" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" t="n">
+        <v>59</v>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>45388</v>
       </c>
-      <c r="G16" t="n">
+      <c r="H16" t="n">
         <v>7</v>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="n">
+        <v>17</v>
+      </c>
+      <c r="J16" t="inlineStr">
         <is>
           <t>条帚门</t>
         </is>
       </c>
-      <c r="I16" t="n">
+      <c r="K16" t="n">
         <v>2</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="L16" t="inlineStr">
         <is>
           <t>Shun Ping 17</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
+      <c r="M16" t="inlineStr">
         <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="L16" t="inlineStr"/>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr"/>
+      <c r="T16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1250,39 +1350,45 @@
         <v>45041</v>
       </c>
       <c r="E17" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F17" t="n">
+        <v>54</v>
+      </c>
+      <c r="G17" s="2" t="n">
         <v>45043</v>
       </c>
-      <c r="G17" t="n">
+      <c r="H17" t="n">
         <v>14</v>
       </c>
-      <c r="H17" t="inlineStr">
+      <c r="I17" t="n">
+        <v>22</v>
+      </c>
+      <c r="J17" t="inlineStr">
         <is>
           <t>虾峙门</t>
         </is>
       </c>
-      <c r="I17" t="n">
+      <c r="K17" t="n">
         <v>2</v>
       </c>
-      <c r="J17" t="inlineStr">
+      <c r="L17" t="inlineStr">
         <is>
           <t>Zhou Shun 10</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="M17" t="inlineStr">
         <is>
           <t>Dong Gang You66</t>
         </is>
       </c>
-      <c r="L17" t="inlineStr"/>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr"/>
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
+      <c r="S17" t="inlineStr"/>
+      <c r="T17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1300,39 +1406,45 @@
         <v>45041</v>
       </c>
       <c r="E18" t="n">
-        <v>8</v>
-      </c>
-      <c r="F18" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F18" t="n">
+        <v>54</v>
+      </c>
+      <c r="G18" s="2" t="n">
         <v>45043</v>
       </c>
-      <c r="G18" t="n">
+      <c r="H18" t="n">
         <v>14</v>
       </c>
-      <c r="H18" t="inlineStr">
+      <c r="I18" t="n">
+        <v>22</v>
+      </c>
+      <c r="J18" t="inlineStr">
         <is>
           <t>虾峙门</t>
         </is>
       </c>
-      <c r="I18" t="n">
+      <c r="K18" t="n">
         <v>2</v>
       </c>
-      <c r="J18" t="inlineStr">
+      <c r="L18" t="inlineStr">
         <is>
           <t>Zhou Shun 10</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
+      <c r="M18" t="inlineStr">
         <is>
           <t>Dong Gang You66</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr"/>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr"/>
       <c r="Q18" t="inlineStr"/>
       <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr"/>
+      <c r="T18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1352,37 +1464,43 @@
       <c r="E19" t="n">
         <v>8</v>
       </c>
-      <c r="F19" s="2" t="n">
+      <c r="F19" t="n">
+        <v>2</v>
+      </c>
+      <c r="G19" s="2" t="n">
         <v>44916</v>
       </c>
-      <c r="G19" t="n">
+      <c r="H19" t="n">
         <v>3</v>
       </c>
-      <c r="H19" t="inlineStr">
+      <c r="I19" t="n">
+        <v>22</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I19" t="n">
+      <c r="K19" t="n">
         <v>2</v>
       </c>
-      <c r="J19" t="inlineStr">
+      <c r="L19" t="inlineStr">
         <is>
           <t>Qi Chen 6</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
+      <c r="M19" t="inlineStr">
         <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr"/>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr"/>
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr"/>
+      <c r="T19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1402,37 +1520,43 @@
       <c r="E20" t="n">
         <v>8</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" t="n">
+        <v>2</v>
+      </c>
+      <c r="G20" s="2" t="n">
         <v>44916</v>
       </c>
-      <c r="G20" t="n">
+      <c r="H20" t="n">
         <v>3</v>
       </c>
-      <c r="H20" t="inlineStr">
+      <c r="I20" t="n">
+        <v>22</v>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>秀山东</t>
         </is>
       </c>
-      <c r="I20" t="n">
+      <c r="K20" t="n">
         <v>2</v>
       </c>
-      <c r="J20" t="inlineStr">
+      <c r="L20" t="inlineStr">
         <is>
           <t>Qi Chen 6</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
+      <c r="M20" t="inlineStr">
         <is>
           <t>Yuan Xiang You 16</t>
         </is>
       </c>
-      <c r="L20" t="inlineStr"/>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr"/>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr"/>
       <c r="Q20" t="inlineStr"/>
       <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr"/>
+      <c r="T20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1452,33 +1576,39 @@
       <c r="E21" t="n">
         <v>14</v>
       </c>
-      <c r="F21" s="2" t="n">
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2" t="n">
         <v>45403</v>
       </c>
-      <c r="G21" t="n">
+      <c r="H21" t="n">
         <v>13</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>虾峙门</t>
-        </is>
       </c>
       <c r="I21" t="n">
         <v>1</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
+          <t>虾峙门</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
           <t>Dong Gang You66</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr"/>
-      <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr"/>
       <c r="Q21" t="inlineStr"/>
       <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr"/>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1498,33 +1628,39 @@
       <c r="E22" t="n">
         <v>14</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2" t="n">
         <v>45403</v>
       </c>
-      <c r="G22" t="n">
+      <c r="H22" t="n">
         <v>13</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>虾峙门</t>
-        </is>
       </c>
       <c r="I22" t="n">
         <v>1</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
+          <t>虾峙门</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>1</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
           <t>Dong Gang You66</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr"/>
-      <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr"/>
       <c r="Q22" t="inlineStr"/>
       <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: use rounded hour for time window matching, remove minute handling
- Use _round datetime for start/end hour extraction in stage 2, ensuring
  consistency with hour-granularity matching in stages 3-4
- Remove start_mins handling in stages 3-4: anchor/weather data are at
  hour granularity, so start_dt should always use :00 minutes
- Update expected coverage values in stage 5 to match corrected
  window sizes (12/24/48)
</commit_message>
<xml_diff>
--- a/logs/duplicate_transactions_real.xlsx
+++ b/logs/duplicate_transactions_real.xlsx
@@ -550,7 +550,7 @@
         <v>44979</v>
       </c>
       <c r="E2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="n">
         <v>35</v>
@@ -606,7 +606,7 @@
         <v>44979</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
         <v>35</v>
@@ -654,7 +654,7 @@
         <v>44979</v>
       </c>
       <c r="E4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" t="n">
         <v>35</v>
@@ -719,7 +719,7 @@
         <v>45028</v>
       </c>
       <c r="H5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I5" t="n">
         <v>41</v>
@@ -775,7 +775,7 @@
         <v>45028</v>
       </c>
       <c r="H6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I6" t="n">
         <v>41</v>
@@ -823,7 +823,7 @@
         <v>45028</v>
       </c>
       <c r="H7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I7" t="n">
         <v>41</v>
@@ -870,7 +870,7 @@
         <v>45065</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>39</v>
@@ -879,7 +879,7 @@
         <v>45066</v>
       </c>
       <c r="H8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I8" t="n">
         <v>39</v>
@@ -922,7 +922,7 @@
         <v>45065</v>
       </c>
       <c r="E9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F9" t="n">
         <v>39</v>
@@ -931,7 +931,7 @@
         <v>45066</v>
       </c>
       <c r="H9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I9" t="n">
         <v>39</v>
@@ -970,7 +970,7 @@
         <v>45065</v>
       </c>
       <c r="E10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F10" t="n">
         <v>39</v>
@@ -979,7 +979,7 @@
         <v>45066</v>
       </c>
       <c r="H10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I10" t="n">
         <v>39</v>
@@ -1022,7 +1022,7 @@
         <v>45403</v>
       </c>
       <c r="E11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F11" t="n">
         <v>44</v>
@@ -1078,7 +1078,7 @@
         <v>45403</v>
       </c>
       <c r="E12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F12" t="n">
         <v>44</v>
@@ -1238,7 +1238,7 @@
         <v>45386</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
         <v>59</v>
@@ -1294,7 +1294,7 @@
         <v>45386</v>
       </c>
       <c r="E16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F16" t="n">
         <v>59</v>
@@ -1350,7 +1350,7 @@
         <v>45041</v>
       </c>
       <c r="E17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F17" t="n">
         <v>54</v>
@@ -1406,7 +1406,7 @@
         <v>45041</v>
       </c>
       <c r="E18" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F18" t="n">
         <v>54</v>

</xml_diff>